<commit_message>
Update data extraction files and add README documentation for reviewers
</commit_message>
<xml_diff>
--- a/03-screening/deduplication-log.xlsx
+++ b/03-screening/deduplication-log.xlsx
@@ -492,13 +492,13 @@
         </is>
       </c>
       <c r="B2" s="2" t="n">
-        <v>658</v>
+        <v>142</v>
       </c>
       <c r="C2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="D2" s="2" t="n">
-        <v>658</v>
+        <v>142</v>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>

</xml_diff>